<commit_message>
Add locale-sensitive GetNumberFormatString for built-in time formats 20 and 21
Extend GetBuiltinNumberFormat(numFmtId, provider) to derive format strings
for built-in indices 20 (h:mm) and 21 (h:mm:ss) from the provider's
ShortTimePattern and LongTimePattern respectively, consistent with how
index 22 already derives its time component.

Also update Issue461.xlsx to include cells with numFmtId 20 and 21,
and add corresponding tests.
</commit_message>
<xml_diff>
--- a/src/TestData/Issue461.xlsx
+++ b/src/TestData/Issue461.xlsx
@@ -35,12 +35,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -61,6 +63,12 @@
       <c r="D1" s="4">
         <v>44927</v>
       </c>
+      <c r="E1" s="5">
+        <v>44927</v>
+      </c>
+      <c r="F1" s="6">
+        <v>44927</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>